<commit_message>
reanalysed hole data for maria
</commit_message>
<xml_diff>
--- a/Compiled Data/merged_afm_data.xlsx
+++ b/Compiled Data/merged_afm_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fb7a53591c131afc/Documents/Summer26/Compiled Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{1EEBAEA9-F0AA-4535-B607-163CF9D1A63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DAB63D-ED56-48F5-A8CA-4A8C88EA74D1}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{1EEBAEA9-F0AA-4535-B607-163CF9D1A63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1354B60-D133-48A6-82B1-F5ECB73C41E1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="107">
   <si>
     <t>Sample ID</t>
   </si>
@@ -3253,6 +3253,12 @@
       <c r="T26" t="s">
         <v>77</v>
       </c>
+      <c r="U26">
+        <v>3.0013809999999999</v>
+      </c>
+      <c r="V26">
+        <v>8.5244E-2</v>
+      </c>
       <c r="W26">
         <v>106</v>
       </c>
@@ -3273,6 +3279,9 @@
       </c>
       <c r="AC26">
         <v>1.1559090000000001</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>70</v>
       </c>
       <c r="AE26" t="s">
         <v>74</v>
@@ -3363,6 +3372,12 @@
       <c r="T27" t="s">
         <v>79</v>
       </c>
+      <c r="U27">
+        <v>6.0826710000000004</v>
+      </c>
+      <c r="V27">
+        <v>2.0291320000000002</v>
+      </c>
       <c r="W27">
         <v>164</v>
       </c>
@@ -3383,6 +3398,9 @@
       </c>
       <c r="AC27">
         <v>5.2805369999999998</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>71</v>
       </c>
       <c r="AE27" t="s">
         <v>73</v>
@@ -3473,6 +3491,12 @@
       <c r="T28" t="s">
         <v>81</v>
       </c>
+      <c r="U28">
+        <v>6.5698030000000003</v>
+      </c>
+      <c r="V28">
+        <v>2.2874569999999999</v>
+      </c>
       <c r="W28">
         <v>463</v>
       </c>
@@ -3493,6 +3517,9 @@
       </c>
       <c r="AC28">
         <v>5.1421419999999998</v>
+      </c>
+      <c r="AD28" t="s">
+        <v>71</v>
       </c>
       <c r="AE28" t="s">
         <v>73</v>
@@ -3583,6 +3610,12 @@
       <c r="T29" t="s">
         <v>84</v>
       </c>
+      <c r="U29">
+        <v>2.9997929999999999</v>
+      </c>
+      <c r="V29">
+        <v>8.7859000000000007E-2</v>
+      </c>
       <c r="W29">
         <v>28</v>
       </c>
@@ -3603,6 +3636,9 @@
       </c>
       <c r="AC29">
         <v>4.6952769999999999</v>
+      </c>
+      <c r="AD29" t="s">
+        <v>70</v>
       </c>
       <c r="AE29" t="s">
         <v>73</v>
@@ -3693,6 +3729,15 @@
       <c r="T30" t="s">
         <v>87</v>
       </c>
+      <c r="U30">
+        <v>5.332217</v>
+      </c>
+      <c r="V30">
+        <v>0.92325500000000005</v>
+      </c>
+      <c r="AD30" t="s">
+        <v>71</v>
+      </c>
       <c r="AE30" t="s">
         <v>70</v>
       </c>
@@ -3767,6 +3812,15 @@
       <c r="T31" t="s">
         <v>90</v>
       </c>
+      <c r="U31">
+        <v>3.9894880000000001</v>
+      </c>
+      <c r="V31">
+        <v>0.41426800000000003</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>71</v>
+      </c>
       <c r="AE31" t="s">
         <v>70</v>
       </c>
@@ -3838,6 +3892,12 @@
       <c r="S32" s="3">
         <v>8.4000000000000005E-2</v>
       </c>
+      <c r="U32">
+        <v>4.6798679999999999</v>
+      </c>
+      <c r="V32">
+        <v>0.96627300000000005</v>
+      </c>
       <c r="W32">
         <v>58</v>
       </c>
@@ -3858,6 +3918,9 @@
       </c>
       <c r="AC32">
         <v>3.6822520000000001</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>71</v>
       </c>
       <c r="AE32" t="s">
         <v>73</v>

</xml_diff>